<commit_message>
feat(F-NAR-019): TREE-DIF-062 passe agent après apply
</commit_message>
<xml_diff>
--- a/stories/arbres/TREE-DIF-062.xlsx
+++ b/stories/arbres/TREE-DIF-062.xlsx
@@ -4221,17 +4221,17 @@
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>On recule. Ils s'éloignent des abeilles, un pas. Près des. Nino attend, les lèvres fermées. Près des pots, le petit. Je l'entends, maintenant. Le seau rouge reste contre la jambe. Le mot est venu, tout seul. Tu as laissé la fin.</t>
+          <t>On recule. Ils s'éloignent des abeilles, un pas. Près des. Nino attend, les lèvres fermées. Près des pots, le petit. Je l'entends, maintenant. Le seau rouge reste contre la jambe. Le mot est venu, tout seul. Le mot était long, cette fois.</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;On recule. Ils s'éloignent des abeilles, un pas. Près des. Nino attend, les lèvres fermées. Près des pots, le petit. Je l'entends, maintenant. Le seau rouge reste contre la jambe. Le mot est venu, tout seul. Tu as laissé la fin.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;On recule. Ils s'éloignent des abeilles, un pas. Près des. Nino attend, les lèvres fermées. Près des pots, le petit. Je l'entends, maintenant. Le seau rouge reste contre la jambe. Le mot est venu, tout seul. Le mot était long, cette fois.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>On recule. Ils s'éloignent des abeilles, un pas. Près des. Nino attend, les lèvres fermées. Près des pots, le petit. Je l'entends, maintenant. Le seau rouge reste contre la jambe. Le mot est venu, tout seul. Tu as laissé la fin. [pause]</t>
+          <t>On recule. Ils s'éloignent des abeilles, un pas. Près des. Nino attend, les lèvres fermées. Près des pots, le petit. Je l'entends, maintenant. Le seau rouge reste contre la jambe. Le mot est venu, tout seul. Le mot était long, cette fois. [pause]</t>
         </is>
       </c>
       <c r="H18" s="2" t="inlineStr"/>
@@ -4373,7 +4373,7 @@
 enfant-m|Je l'entends, maintenant.
 narrateur|Le seau rouge reste contre la jambe.
 maman|Le mot est venu, tout seul.
-papa|Tu as laissé la fin.</t>
+papa|Le mot était long, cette fois.</t>
         </is>
       </c>
       <c r="AX18" t="inlineStr">
@@ -15056,17 +15056,17 @@
       </c>
       <c r="E76" s="2" t="inlineStr">
         <is>
-          <t>Mes mains, et le torchon. Une main écoute, l'autre tient le linge. Le bourdon s'éloigne, un peu. Près des. Nino ne frotte pas trop tôt. Près des feuilles. Le torchon dort contre sa poche. Tes mains ont deux métiers. Écouter d'abord, essuyer après.</t>
+          <t>Mes mains, et le torchon. Une main écoute, l'autre tient le linge. Le bourdon s'éloigne, un peu. Près des. Nino ne frotte pas trop tôt. Près des feuilles. Le torchon dort contre sa poche. Tes mains ont deux métiers. Le linge peut attendre, un peu.</t>
         </is>
       </c>
       <c r="F76" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Mes mains, et le torchon. Une main écoute, l'autre tient le linge. Le bourdon s'éloigne, un peu. Près des. Nino ne frotte pas trop tôt. Près des feuilles. Le torchon dort contre sa poche. Tes mains ont deux métiers. Écouter d'abord, essuyer après.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Mes mains, et le torchon. Une main écoute, l'autre tient le linge. Le bourdon s'éloigne, un peu. Près des. Nino ne frotte pas trop tôt. Près des feuilles. Le torchon dort contre sa poche. Tes mains ont deux métiers. Le linge peut attendre, un peu.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G76" s="2" t="inlineStr">
         <is>
-          <t>Mes mains, et le torchon. Une main écoute, l'autre tient le linge. Le bourdon s'éloigne, un peu. Près des. Nino ne frotte pas trop tôt. Près des feuilles. Le torchon dort contre sa poche. Tes mains ont deux métiers. Écouter d'abord, essuyer après. [pause]</t>
+          <t>Mes mains, et le torchon. Une main écoute, l'autre tient le linge. Le bourdon s'éloigne, un peu. Près des. Nino ne frotte pas trop tôt. Près des feuilles. Le torchon dort contre sa poche. Tes mains ont deux métiers. Le linge peut attendre, un peu. [pause]</t>
         </is>
       </c>
       <c r="H76" s="2" t="inlineStr"/>
@@ -15208,7 +15208,7 @@
 maman|Près des feuilles.
 narrateur|Le torchon dort contre sa poche.
 papa|Tes mains ont deux métiers.
-maman|Écouter d'abord, essuyer après.</t>
+maman|Le linge peut attendre, un peu.</t>
         </is>
       </c>
       <c r="AX76" t="inlineStr">
@@ -15425,17 +15425,17 @@
       </c>
       <c r="E78" s="2" t="inlineStr">
         <is>
-          <t>Le banc, le torchon sur les genoux. On s'assoit, le thym est là. Le tissu attend, plié, sans bouger. Le petit pot. Nino lève le torchon, après le mot. Je l'essuie, contre le thym. Le torchon dort contre sa poche. Le banc a gardé le linge. Le mot d'abord, le tissu ensuite.</t>
+          <t>Le banc, le torchon sur les genoux. On s'assoit, le thym est là. Le tissu attend, plié, sans bouger. Le petit pot. Nino lève le torchon, après le mot. Je l'essuie, contre le thym. Le torchon dort contre sa poche. Le banc a gardé le linge. Le thym a eu son mot, puis le linge.</t>
         </is>
       </c>
       <c r="F78" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le &lt;emphasis level="moderate"&gt;banc&lt;/emphasis&gt;, le torchon sur les genoux. On s'assoit, le thym est là. Le tissu attend, plié, sans bouger. Le petit pot. Nino lève le torchon, après le mot. Je l'essuie, contre le thym. Le torchon dort contre sa poche. Le banc a gardé le linge. Le mot d'abord, le tissu ensuite.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le &lt;emphasis level="moderate"&gt;banc&lt;/emphasis&gt;, le torchon sur les genoux. On s'assoit, le thym est là. Le tissu attend, plié, sans bouger. Le petit pot. Nino lève le torchon, après le mot. Je l'essuie, contre le thym. Le torchon dort contre sa poche. Le banc a gardé le linge. Le thym a eu son mot, puis le linge.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G78" s="2" t="inlineStr">
         <is>
-          <t>Le &lt;emphasis&gt;banc&lt;/emphasis&gt;, le torchon sur les genoux. On s'assoit, le thym est là. Le tissu attend, plié, sans bouger. Le petit pot. Nino lève le torchon, après le mot. Je l'essuie, contre le thym. Le torchon dort contre sa poche. Le banc a gardé le linge. Le mot d'abord, le tissu ensuite. [pause]</t>
+          <t>Le &lt;emphasis&gt;banc&lt;/emphasis&gt;, le torchon sur les genoux. On s'assoit, le thym est là. Le tissu attend, plié, sans bouger. Le petit pot. Nino lève le torchon, après le mot. Je l'essuie, contre le thym. Le torchon dort contre sa poche. Le banc a gardé le linge. Le thym a eu son mot, puis le linge. [pause]</t>
         </is>
       </c>
       <c r="H78" s="2" t="inlineStr"/>
@@ -15577,7 +15577,7 @@
 enfant-m|Je l'essuie, contre le thym.
 narrateur|Le torchon dort contre sa poche.
 papa|Le banc a gardé le linge.
-maman|Le mot d'abord, le tissu ensuite.</t>
+maman|Le thym a eu son mot, puis le linge.</t>
         </is>
       </c>
       <c r="AX78" t="inlineStr">
@@ -17281,7 +17281,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A16"/>
+  <dimension ref="A1:A17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -17394,6 +17394,13 @@
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>